<commit_message>
docs: add BLE MIDI and D1 core roadmap
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rdd19fbb7426d49e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R3d8ccb4094e7426a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R4379077619f64dfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rd65e7e5093f54f4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R72ded0b324cc43bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Re84e7d5b1aa24452"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R7f934b418b894390"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R9a7473e9a57b46bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rd84424c244d844a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R66e43e1e915b496a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R3faf841bc6b649af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R4c35feeb56314f52"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -245,7 +245,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="83">
+  <x:cellXfs count="84">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -435,6 +435,9 @@
     <x:xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="16" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="16" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -513,8 +516,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogTable" displayName="BacklogTable" ref="A4:L65" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:L65"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogTable" displayName="BacklogTable" ref="A4:L67" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:L67"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Story ID"/>
     <x:tableColumn id="2" name="Epic"/>
@@ -548,7 +551,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RisksTable" displayName="RisksTable" ref="A4:G26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RisksTable" displayName="RisksTable" ref="A4:G29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risiko"/>
@@ -574,7 +577,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Bron"/>
     <x:tableColumn id="2" name="Gebruik"/>
@@ -804,7 +807,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="52" t="str">
-        <x:v>Sprint 1 | v0.3.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 1 | scope v0.4.0 | runtime v0.3.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="51"/>
       <x:c r="C2" s="51"/>
@@ -845,8 +848,8 @@
         <x:v>Totale stories</x:v>
       </x:c>
       <x:c r="B5" s="57" t="n">
-        <x:f>COUNTA('Backlog'!$A$5:$A$65)</x:f>
-        <x:v>61</x:v>
+        <x:f>COUNTA('Backlog'!$A$5:$A$67)</x:f>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C5" s="51"/>
       <x:c r="D5" s="56" t="str">
@@ -862,7 +865,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B6" s="59" t="n">
-        <x:f>COUNTIF('Backlog'!$F$5:$F$65,"Done")</x:f>
+        <x:f>COUNTIF('Backlog'!$F$5:$F$67,"Done")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C6" s="51"/>
@@ -879,12 +882,12 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B7" s="59" t="n">
-        <x:f>COUNTIF('Backlog'!$F$5:$F$65,"In Progress")</x:f>
+        <x:f>COUNTIF('Backlog'!$F$5:$F$67,"In Progress")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="51"/>
       <x:c r="D7" s="58" t="str">
-        <x:v>3. Standalone host/DIN-transport moet sonder DAW slaag</x:v>
+        <x:v>3. D1-basiskern voor SN76489; SID en OPL daarna</x:v>
       </x:c>
       <x:c r="E7" s="58"/>
       <x:c r="F7" s="58"/>
@@ -896,12 +899,12 @@
         <x:v>MVP-gemerk</x:v>
       </x:c>
       <x:c r="B8" s="59" t="n">
-        <x:f>COUNTIF('Backlog'!$E$5:$E$65,"Must")</x:f>
-        <x:v>44</x:v>
+        <x:f>COUNTIF('Backlog'!$E$5:$E$67,"Must")</x:f>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C8" s="51"/>
       <x:c r="D8" s="60" t="str">
-        <x:v>4. Twee verskillende kerne eers na een-kern-bewys en resource gate</x:v>
+        <x:v>4. BLE op tweede bord; S2 faal veilig; multi-core na resource gate</x:v>
       </x:c>
       <x:c r="E8" s="60"/>
       <x:c r="F8" s="60"/>
@@ -913,8 +916,8 @@
         <x:v>Oop risiko’s</x:v>
       </x:c>
       <x:c r="B9" s="59" t="n">
-        <x:f>COUNTIF('Risks'!$G$5:$G$26,"&lt;&gt;Closed")</x:f>
-        <x:v>22</x:v>
+        <x:f>COUNTIF('Risks'!$G$5:$G$29,"&lt;&gt;Closed")</x:f>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C9" s="51"/>
       <x:c r="D9" s="51"/>
@@ -1053,7 +1056,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md | 61 stories | Redigeer Status en Priority via keuselyste</x:v>
+        <x:v>Bron: docs/user_stories_v0.1.0.md | 63 stories | Redigeer Status en Priority via keuselyste</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -1731,10 +1734,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J21" s="24" t="str">
-        <x:v>US-006, US-014</x:v>
+        <x:v>US-063</x:v>
       </x:c>
       <x:c r="K21" s="24" t="str">
-        <x:v>Drie toonstemme speel onafhanklik met gedokumenteerde akkuraatheid</x:v>
+        <x:v>Tweede musikale kern: drie toonstemme speel onafhanklik met gedokumenteerde akkuraatheid</x:v>
       </x:c>
       <x:c r="L21" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-017</x:v>
@@ -1845,7 +1848,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J24" s="24" t="str">
-        <x:v>US-015, US-017</x:v>
+        <x:v>US-016, US-063</x:v>
       </x:c>
       <x:c r="K24" s="24" t="str">
         <x:v>Opsionele sestiendenootreeks bewys die klankpad by start</x:v>
@@ -3046,7 +3049,7 @@
         <x:v>QA/Release</x:v>
       </x:c>
       <x:c r="E56" s="24" t="str">
-        <x:v>Should</x:v>
+        <x:v>Must</x:v>
       </x:c>
       <x:c r="F56" s="24" t="str">
         <x:v>Backlog</x:v>
@@ -3055,7 +3058,7 @@
         <x:v>Release train</x:v>
       </x:c>
       <x:c r="H56" s="24" t="str">
-        <x:v>Later</x:v>
+        <x:v>MVP</x:v>
       </x:c>
       <x:c r="I56" s="65" t="n">
         <x:v>8</x:v>
@@ -3064,7 +3067,7 @@
         <x:v>US-004</x:v>
       </x:c>
       <x:c r="K56" s="24" t="str">
-        <x:v>’n tweede CircuitPython-mikrobeheerder werk via ’n profiel</x:v>
+        <x:v>'n Tweede BLE-geskikte CircuitPython-mikrobeheerder werk via 'n profiel sonder S2-regressie</x:v>
       </x:c>
       <x:c r="L56" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-052</x:v>
@@ -3410,6 +3413,82 @@
       </x:c>
       <x:c r="L65" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MIDI-TRANSPORT-MULTICORE-AMENDMENT-001 / MCP-US-061</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="48" customHeight="1">
+      <x:c r="A66" s="83" t="str">
+        <x:v>MCP-US-062</x:v>
+      </x:c>
+      <x:c r="B66" s="83" t="str">
+        <x:v>MCP-EPIC-002</x:v>
+      </x:c>
+      <x:c r="C66" s="83" t="str">
+        <x:v>BLE MIDI Transport And Capability Gate</x:v>
+      </x:c>
+      <x:c r="D66" s="83" t="str">
+        <x:v>MIDI Engineer</x:v>
+      </x:c>
+      <x:c r="E66" s="83" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="F66" s="83" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G66" s="83" t="str">
+        <x:v>Sprint 4</x:v>
+      </x:c>
+      <x:c r="H66" s="83" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="I66" s="83" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J66" s="83" t="str">
+        <x:v>US-006, US-007, US-052</x:v>
+      </x:c>
+      <x:c r="K66" s="83" t="str">
+        <x:v>BLE-bord ontvang Note/CC/bend via dieselfde eventmodel; S2 rapporteer unsupported sonder USB-regressie</x:v>
+      </x:c>
+      <x:c r="L66" s="83" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / SCOPE-AMENDMENT-002 / MCP-US-062</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="48" customHeight="1">
+      <x:c r="A67" s="83" t="str">
+        <x:v>MCP-US-063</x:v>
+      </x:c>
+      <x:c r="B67" s="83" t="str">
+        <x:v>MCP-EPIC-003</x:v>
+      </x:c>
+      <x:c r="C67" s="83" t="str">
+        <x:v>Portable D1 Baseline Synth Core</x:v>
+      </x:c>
+      <x:c r="D67" s="83" t="str">
+        <x:v>DSP/Chip Engineer</x:v>
+      </x:c>
+      <x:c r="E67" s="83" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="F67" s="83" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G67" s="83" t="str">
+        <x:v>Sprint 3</x:v>
+      </x:c>
+      <x:c r="H67" s="83" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="I67" s="83" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J67" s="83" t="str">
+        <x:v>US-006, US-014, US-016</x:v>
+      </x:c>
+      <x:c r="K67" s="83" t="str">
+        <x:v>Nuut-geporteerde sine/saw/square D1-gedrag speel via AudioOutput; geen desktop-backend of produksierepo-wysiging</x:v>
+      </x:c>
+      <x:c r="L67" s="83" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / SCOPE-AMENDMENT-002 / MCP-US-063</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3425,7 +3504,7 @@
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Ready"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="4">
+  <x:dataValidations count="6">
     <x:dataValidation type="list" sqref="E5:E61">
       <x:formula1>"Must,Should,Could,Won't now"</x:formula1>
     </x:dataValidation>
@@ -3438,10 +3517,16 @@
     <x:dataValidation type="list" sqref="F62:F63">
       <x:formula1>"Backlog,Ready,In Progress,Review,Done,Impediment"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="E66:E67">
+      <x:formula1>"Must,Should,Could,Won't now"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F66:F67">
+      <x:formula1>"Backlog,In Progress,In Review,Done,Blocked"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9656ca5643894423"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fcd065b88be4856"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3496,15 +3581,15 @@
         <x:v>Platform Foundation</x:v>
       </x:c>
       <x:c r="C5" s="64" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A5)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A5)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D5" s="64" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A5,'Backlog'!$E$5:$E$65,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A5,'Backlog'!$E$5:$E$67,"Must")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E5" s="64" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A5,'Backlog'!$F$5:$F$65,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A5,'Backlog'!$F$5:$F$67,"Done")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="F5" s="23" t="str">
@@ -3519,19 +3604,19 @@
         <x:v>MIDI And Clock</x:v>
       </x:c>
       <x:c r="C6" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A6)</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A6)</x:f>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D6" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A6,'Backlog'!$E$5:$E$65,"Must")</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A6,'Backlog'!$E$5:$E$67,"Must")</x:f>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E6" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A6,'Backlog'!$F$5:$F$65,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A6,'Backlog'!$F$5:$F$67,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="24" t="str">
-        <x:v>USB-MIDI, guitar slides, kontroles en interne/eksterne klok</x:v>
+        <x:v>USB, BLE en DIN/UART MIDI; guitar slides, kontroles en clock</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="32" customHeight="1">
@@ -3542,19 +3627,19 @@
         <x:v>Audio And Chip Core</x:v>
       </x:c>
       <x:c r="C7" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A7)</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A7)</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D7" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A7,'Backlog'!$E$5:$E$65,"Must")</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A7,'Backlog'!$E$5:$E$67,"Must")</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E7" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A7,'Backlog'!$F$5:$F$65,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A7,'Backlog'!$F$5:$F$67,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
-        <x:v>MAX98357 mono eerste, SN76489 en latere stereo</x:v>
+        <x:v>MAX98357 mono eerste; D1-basiskern, SN76489 en latere stereo</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
@@ -3565,15 +3650,15 @@
         <x:v>Local Web Control</x:v>
       </x:c>
       <x:c r="C8" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A8)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A8)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D8" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A8,'Backlog'!$E$5:$E$65,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A8,'Backlog'!$E$5:$E$67,"Must")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="E8" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A8,'Backlog'!$F$5:$F$65,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A8,'Backlog'!$F$5:$F$67,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F8" s="24" t="str">
@@ -3588,15 +3673,15 @@
         <x:v>Files, Harmony And Performance Tools</x:v>
       </x:c>
       <x:c r="C9" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A9)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A9)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D9" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A9,'Backlog'!$E$5:$E$65,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A9,'Backlog'!$E$5:$E$67,"Must")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E9" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A9,'Backlog'!$F$5:$F$65,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A9,'Backlog'!$F$5:$F$67,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="24" t="str">
@@ -3611,15 +3696,15 @@
         <x:v>Multi-Core Expansion</x:v>
       </x:c>
       <x:c r="C10" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A10)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A10)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D10" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A10,'Backlog'!$E$5:$E$65,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A10,'Backlog'!$E$5:$E$67,"Must")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E10" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A10,'Backlog'!$F$5:$F$65,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A10,'Backlog'!$F$5:$F$67,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F10" s="24" t="str">
@@ -3634,15 +3719,15 @@
         <x:v>DSP And Pedal Hardware</x:v>
       </x:c>
       <x:c r="C11" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A11)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A11)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D11" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A11,'Backlog'!$E$5:$E$65,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A11,'Backlog'!$E$5:$E$67,"Must")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="E11" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A11,'Backlog'!$F$5:$F$65,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A11,'Backlog'!$F$5:$F$67,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="24" t="str">
@@ -3657,19 +3742,19 @@
         <x:v>Portability, Quality And Release</x:v>
       </x:c>
       <x:c r="C12" s="66" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A12)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A12)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D12" s="66" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A12,'Backlog'!$E$5:$E$65,"Must")</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A12,'Backlog'!$E$5:$E$67,"Must")</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E12" s="66" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A12,'Backlog'!$F$5:$F$65,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A12,'Backlog'!$F$5:$F$67,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F12" s="25" t="str">
-        <x:v>Host/HIL, kruisplatform en release</x:v>
+        <x:v>Host/HIL, BLE-tweedebord, kruisplatform en release</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3679,7 +3764,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1596364ed85242d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59263cba85894f0a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3704,7 +3789,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>22 aktiewe risiko's; hoe risiko's word vroeg sigbaar gemaak en geen demo-status verberg 'n blocker nie</x:v>
+        <x:v>25 aktiewe risiko's; blockers bly sigbaar en firmwarebewys word van hosttooling onderskei</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -4213,26 +4298,95 @@
         <x:v>Controlled</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="40" customHeight="1">
-      <x:c r="A26" t="str">
+    <x:row r="26" ht="48" customHeight="1">
+      <x:c r="A26" s="83" t="str">
         <x:v>R-022</x:v>
       </x:c>
-      <x:c r="B26" t="str">
-        <x:v>MIDI-HIL hang deur poortkonflik met Thonny of serial monitor</x:v>
-      </x:c>
-      <x:c r="C26" t="str">
+      <x:c r="B26" s="83" t="str">
+        <x:v>Eksterne USB-host ondersteun nie die betrokke controller of bend/clock-boodskap nie</x:v>
+      </x:c>
+      <x:c r="C26" s="83" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="D26" t="str">
+      <x:c r="D26" s="83" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="E26" t="str">
+      <x:c r="E26" s="83" t="str">
+        <x:v>MIDI/QA</x:v>
+      </x:c>
+      <x:c r="F26" s="83" t="str">
+        <x:v>Compatibility matrix; generiese plus Fishman HIL; geen handelsnaamwaarborg sonder toets nie</x:v>
+      </x:c>
+      <x:c r="G26" s="83" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="48" customHeight="1">
+      <x:c r="A27" s="83" t="str">
+        <x:v>R-023</x:v>
+      </x:c>
+      <x:c r="B27" s="83" t="str">
+        <x:v>BLE-MIDI is Must, maar die primere ESP32-S2 het geen native BLE nie</x:v>
+      </x:c>
+      <x:c r="C27" s="83" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D27" s="83" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E27" s="83" t="str">
+        <x:v>Architect/Embedded</x:v>
+      </x:c>
+      <x:c r="F27" s="83" t="str">
+        <x:v>Capability gate; tweede BLE-bordprofiel in US-052 en positiewe HIL in US-062</x:v>
+      </x:c>
+      <x:c r="G27" s="83" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="48" customHeight="1">
+      <x:c r="A28" s="83" t="str">
+        <x:v>R-024</x:v>
+      </x:c>
+      <x:c r="B28" s="83" t="str">
+        <x:v>Herhaalde macOS host-MIDI-scan abort in python-rtmidi/CoreMIDI</x:v>
+      </x:c>
+      <x:c r="C28" s="83" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D28" s="83" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="E28" s="83" t="str">
+        <x:v>QA/Tooling</x:v>
+      </x:c>
+      <x:c r="F28" s="83" t="str">
+        <x:v>Geen herhaalde in-proses scan; toekomstige host-scan in subprocess; device logs vir firmware-HIL</x:v>
+      </x:c>
+      <x:c r="G28" s="83" t="str">
+        <x:v>Open - host impediment</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="48" customHeight="1">
+      <x:c r="A29" s="83" t="str">
+        <x:v>R-025</x:v>
+      </x:c>
+      <x:c r="B29" s="83" t="str">
+        <x:v>MIDI-HIL hang of faal deur poortkonflik met Thonny of serial monitor</x:v>
+      </x:c>
+      <x:c r="C29" s="83" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="D29" s="83" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E29" s="83" t="str">
         <x:v>QA/HIL</x:v>
       </x:c>
-      <x:c r="F26" t="str">
-        <x:v>Preflight lsof; een REPL-klient; timeout en herstelpad</x:v>
-      </x:c>
-      <x:c r="G26" t="str">
+      <x:c r="F29" s="83" t="str">
+        <x:v>Preflight poorte; een REPL-klient; timeout, cleanup en herstelpad</x:v>
+      </x:c>
+      <x:c r="G29" s="83" t="str">
         <x:v>Open</x:v>
       </x:c>
     </x:row>
@@ -4247,17 +4401,20 @@
   <x:conditionalFormatting sqref="G5:G22">
     <x:cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="Closed"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="G5:G22">
       <x:formula1>"Open,Open - human action,Controlled,Closed"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="G23">
       <x:formula1>"Open,Controlled,Open - human action,Closed"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="G27:G29">
+      <x:formula1>"Open,Controlled,Closed,Open - human action,Open - host impediment"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3f34a4217444cb0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R692321d367e54e0f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4431,7 +4588,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ff325af1a474206"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69b9c7dfc5ca4a9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4708,6 +4865,62 @@
         <x:v>https://github.com/rppicomidi/RasPiMIDIHub</x:v>
       </x:c>
     </x:row>
+    <x:row r="22" ht="38" customHeight="1">
+      <x:c r="A22" s="83" t="str">
+        <x:v>CircuitPython _bleio</x:v>
+      </x:c>
+      <x:c r="B22" s="83" t="str">
+        <x:v>Native BLE capability en eksplisiete ESP32-S2-uitsondering</x:v>
+      </x:c>
+      <x:c r="C22" s="83" t="str">
+        <x:v>Official API</x:v>
+      </x:c>
+      <x:c r="D22" s="83" t="str">
+        <x:v>https://docs.circuitpython.org/en/latest/shared-bindings/_bleio/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="38" customHeight="1">
+      <x:c r="A23" s="83" t="str">
+        <x:v>Adafruit BLE MIDI</x:v>
+      </x:c>
+      <x:c r="B23" s="83" t="str">
+        <x:v>BLE MIDI service en dependencies</x:v>
+      </x:c>
+      <x:c r="C23" s="83" t="str">
+        <x:v>Official library</x:v>
+      </x:c>
+      <x:c r="D23" s="83" t="str">
+        <x:v>https://docs.circuitpython.org/projects/ble_midi/en/latest/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="38" customHeight="1">
+      <x:c r="A24" s="83" t="str">
+        <x:v>Adafruit BLE MIDI API</x:v>
+      </x:c>
+      <x:c r="B24" s="83" t="str">
+        <x:v>MIDIService as PortIn/PortOut-agtige transport</x:v>
+      </x:c>
+      <x:c r="C24" s="83" t="str">
+        <x:v>Official API</x:v>
+      </x:c>
+      <x:c r="D24" s="83" t="str">
+        <x:v>https://docs.circuitpython.org/projects/ble_midi/en/stable/api.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="38" customHeight="1">
+      <x:c r="A25" s="83" t="str">
+        <x:v>Espressif ESP32-S2 datasheet</x:v>
+      </x:c>
+      <x:c r="B25" s="83" t="str">
+        <x:v>S2 Wi-Fi, USB, I2S en geheuevermoens</x:v>
+      </x:c>
+      <x:c r="C25" s="83" t="str">
+        <x:v>Official datasheet</x:v>
+      </x:c>
+      <x:c r="D25" s="83" t="str">
+        <x:v>https://documentation.espressif.com/esp32-s2_datasheet_en.html</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -4715,7 +4928,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8f3f988567f4c48"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60bfdda777b54386"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add board capability discovery
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb2efe85f9cbd4749"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R49532a6b7ffe47f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rdf74317939d84a63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rf5c1d196cb3948ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Re57d9c22986c46f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R8df0036d754a48fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf8ea33ce5d1c4875"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R218347a9a4ce4b36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Ra5aed93ce89b4521"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Re6f121bba1ad469a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R0f24e0d0a64f47fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R0618949d4d274095"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -551,7 +551,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RisksTable" displayName="RisksTable" ref="A4:G31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RisksTable" displayName="RisksTable" ref="A4:G32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risiko"/>
@@ -577,7 +577,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Bron"/>
     <x:tableColumn id="2" name="Gebruik"/>
@@ -807,7 +807,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="52" t="str">
-        <x:v>Sprint 1 | scope v0.5.0 | runtime v0.3.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 1 | scope v0.6.0 | runtime v0.4.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="51"/>
       <x:c r="C2" s="51"/>
@@ -883,7 +883,7 @@
       </x:c>
       <x:c r="B7" s="59" t="n">
         <x:f>COUNTIF('Backlog'!$F$5:$F$67,"In Progress")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="51"/>
       <x:c r="D7" s="58" t="str">
@@ -916,8 +916,8 @@
         <x:v>Oop risiko’s</x:v>
       </x:c>
       <x:c r="B9" s="59" t="n">
-        <x:f>COUNTIF('Risks'!$G$5:$G$31,"&lt;&gt;Closed")</x:f>
-        <x:v>27</x:v>
+        <x:f>COUNTA('Risks'!A5:A32)</x:f>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C9" s="51"/>
       <x:c r="D9" s="51" t="str">
@@ -965,7 +965,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="62" t="str">
-        <x:v>Aktiewe story: MCP-US-051 Hardware-In-The-Loop Test Runner</x:v>
+        <x:v>Aktiewe story: MCP-US-004 Board Capability Discovery - IMPEDIMENT</x:v>
       </x:c>
       <x:c r="B13" s="51"/>
       <x:c r="C13" s="51"/>
@@ -1230,13 +1230,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F8" s="24" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>Impediment</x:v>
       </x:c>
       <x:c r="G8" s="24" t="str">
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H8" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>In Review/MVP</x:v>
       </x:c>
       <x:c r="I8" s="65" t="n">
         <x:v>5</x:v>
@@ -1245,10 +1245,10 @@
         <x:v>US-002</x:v>
       </x:c>
       <x:c r="K8" s="24" t="str">
-        <x:v>Bordprofiel rapporteer penne, modules, geheue en ondersteunde klankbackends</x:v>
+        <x:v>Host en sagte device-run rapporteer IO3/5/7, modules, heap en I2S-backend; finale hard-reset/remount-HIL wag</x:v>
       </x:c>
       <x:c r="L8" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-004</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-004 / v0.4.0</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="38" customHeight="1">
@@ -3016,13 +3016,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F55" s="24" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="G55" s="24" t="str">
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H55" s="24" t="str">
-        <x:v>In Progress/MVP</x:v>
+        <x:v>In Review/MVP</x:v>
       </x:c>
       <x:c r="I55" s="65" t="n">
         <x:v>5</x:v>
@@ -3506,7 +3506,7 @@
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Ready"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="6">
+  <x:dataValidations count="7">
     <x:dataValidation type="list" sqref="E5:E61">
       <x:formula1>"Must,Should,Could,Won't now"</x:formula1>
     </x:dataValidation>
@@ -3525,10 +3525,13 @@
     <x:dataValidation type="list" sqref="F66:F67">
       <x:formula1>"Backlog,In Progress,In Review,Done,Blocked"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="F5:F67">
+      <x:formula1>"Backlog,Ready,In Progress,Impediment,In Review,Done"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1300f31f2214263"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c96d68be8d0425f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3766,7 +3769,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8b44bac04f54ea3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75f6590912004891"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3791,7 +3794,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>27 aktiewe risiko's; Wi-Fi-fallback en logging bly begrens sonder om real-time klank te verberg</x:v>
+        <x:v>28 aktiewe risiko's; MCP-US-004 is geblokkeer op USB-remount ná programmatiese harde reset</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -3926,10 +3929,10 @@
         <x:v>Embedded</x:v>
       </x:c>
       <x:c r="F9" s="24" t="str">
-        <x:v>Capability profile, MAX98357 HIL en PWM fallback</x:v>
+        <x:v>US-004 bevestig IO5/IO3/IO7 en audiobusio; MAX98357 klank-HIL volg in US-016</x:v>
       </x:c>
       <x:c r="G9" s="24" t="str">
-        <x:v>Open</x:v>
+        <x:v>Controlled</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
@@ -4436,6 +4439,29 @@
       </x:c>
       <x:c r="G31" s="83" t="str">
         <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="44" customHeight="1">
+      <x:c r="A32" s="83" t="str">
+        <x:v>R-028</x:v>
+      </x:c>
+      <x:c r="B32" s="83" t="str">
+        <x:v>Programmatiese harde reset laat USB sonder CIRCUITPY/CDC-herenumerasie</x:v>
+      </x:c>
+      <x:c r="C32" s="83" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="D32" s="83" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E32" s="83" t="str">
+        <x:v>Embedded/QA</x:v>
+      </x:c>
+      <x:c r="F32" s="83" t="str">
+        <x:v>Fisiese power-cycle; recovery-runbook; blokkeer story tot volume, REPL, bootbanner en manifest-HIL herstel</x:v>
+      </x:c>
+      <x:c r="G32" s="83" t="str">
+        <x:v>Open - US-004 impediment</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4465,7 +4491,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Race08dc751e245b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra803290166854d9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4639,7 +4665,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1a6529c66aa4743"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a9a1fadc3dd464f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5000,6 +5026,34 @@
         <x:v>https://docs.circuitpython.org/projects/httpserver/en/latest/starting_methods.html</x:v>
       </x:c>
     </x:row>
+    <x:row r="28" ht="56" customHeight="1">
+      <x:c r="A28" t="str">
+        <x:v>WEMOS S2 Mini</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>Verwysingsbord, 3.3 V-logika, 27 I/O, flash en PSRAM</x:v>
+      </x:c>
+      <x:c r="C28" s="83" t="str">
+        <x:v>Official board documentation</x:v>
+      </x:c>
+      <x:c r="D28" s="83" t="str">
+        <x:v>https://docs.wemos.cc/en/latest/s2/s2_mini.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="56" customHeight="1">
+      <x:c r="A29" t="str">
+        <x:v>Espressif ESP32-S2 I2S</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>Een I2S-perifeer en BCLK/WS/DOUT-semantiek</x:v>
+      </x:c>
+      <x:c r="C29" s="83" t="str">
+        <x:v>Official silicon/driver documentation</x:v>
+      </x:c>
+      <x:c r="D29" s="83" t="str">
+        <x:v>https://docs.espressif.com/projects/esp-idf/en/release-v5.2/esp32s2/api-reference/peripherals/i2s.html</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -5007,7 +5061,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd080a18d380a45fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ae7da3a3867460a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add pitch bend and CC1 control state
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc98236d4d4bd4f43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R1033548ef4544838"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Re367758b5bca48b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R0ac69ad9eaab444d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R7af068346dd94d37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R0b640df49e454752"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R015eca3c5ae74f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R8289e600bf5b4c7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rce8f7e1e88894285"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rcbe5280a3ef84e7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Ra56ed1de19954598"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rb5c5ef7e31b64058"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -980,7 +980,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 2 | scope v0.8.0 | runtime v0.6.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 2 | scope v0.13.0 | runtime v0.11.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1039,7 +1039,7 @@
       </x:c>
       <x:c r="B6" s="114" t="n">
         <x:f>COUNTIF('Backlog'!$F$5:$F$67,"Done")</x:f>
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
@@ -1138,7 +1138,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>Aktiewe story: MCP-US-006 Portable Event Model - IN REVIEW | US-005 HIL HEK OOP | Volgende plan: MCP-US-007</x:v>
+        <x:v>Aktiewe hek: MCP-US-010 hoorbare bend/CC1 wag op I2S + D1 core | US-062 BLE HIL impediment | 68 hosttoetse groen</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1160,7 +1160,7 @@
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" s="123" t="str">
-        <x:v>Product Owner note: hierdie workbook is die redigeerbare Kanban-artefak. Die Markdown story-katalogus bly die leesbare repository-weergawe. Werk begin eers ná story-plan-goedkeuring.</x:v>
+        <x:v>Product Owner note: outonome hoststories is gepush. Fisiese USB/BLE/klank-aanvaarding bly menslike HIL en word nie uit hosttoetse afgelei nie.</x:v>
       </x:c>
       <x:c r="B15" s="124"/>
       <x:c r="C15" s="124"/>
@@ -1517,13 +1517,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F11" s="24" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="G11" s="24" t="str">
         <x:v>Sprint 2</x:v>
       </x:c>
       <x:c r="H11" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="I11" s="65" t="n">
         <x:v>5</x:v>
@@ -1532,10 +1532,10 @@
         <x:v>US-003, US-006</x:v>
       </x:c>
       <x:c r="K11" s="24" t="str">
-        <x:v>Enige klas-kompatibele bron kan via 'n rekenaar/DAW of eksterne USB-host Note On/Off stuur sonder toestelnaamkonstante</x:v>
+        <x:v>Host receive-loop groen; fisiese USB-MIDI Note On/Off wag op herstelbare toestel-deploy</x:v>
       </x:c>
       <x:c r="L11" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007 / commit 3ffc1bc</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
@@ -1555,13 +1555,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F12" s="24" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G12" s="24" t="str">
         <x:v>Sprint 2</x:v>
       </x:c>
       <x:c r="H12" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I12" s="65" t="n">
         <x:v>5</x:v>
@@ -1570,10 +1570,10 @@
         <x:v>US-007</x:v>
       </x:c>
       <x:c r="K12" s="24" t="str">
-        <x:v>Kanaal 1-16 word konfigureerbaar na ’n kerninstansie gerouteer</x:v>
+        <x:v>Kanaal 1-16 roeteer dinamies; kanaallose clock en onbekende kanale bly ongebonde</x:v>
       </x:c>
       <x:c r="L12" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-008</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-008 / commit 68f4dd4</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="38" customHeight="1">
@@ -1593,13 +1593,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F13" s="24" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G13" s="24" t="str">
         <x:v>Sprint 2</x:v>
       </x:c>
       <x:c r="H13" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I13" s="65" t="n">
         <x:v>5</x:v>
@@ -1608,10 +1608,10 @@
         <x:v>US-007</x:v>
       </x:c>
       <x:c r="K13" s="24" t="str">
-        <x:v>Velocity nul sluit note; geen hangende stem ná All Notes Off nie</x:v>
+        <x:v>Velocity nul, Note Off, CC120 en CC123 ruim aktiewe note per kanaal op</x:v>
       </x:c>
       <x:c r="L13" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-009</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-009 / commit 3236850</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="38" customHeight="1">
@@ -1631,13 +1631,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F14" s="24" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="G14" s="24" t="str">
         <x:v>Sprint 2</x:v>
       </x:c>
       <x:c r="H14" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Control ready / audible blocked</x:v>
       </x:c>
       <x:c r="I14" s="65" t="n">
         <x:v>5</x:v>
@@ -1646,10 +1646,10 @@
         <x:v>US-007</x:v>
       </x:c>
       <x:c r="K14" s="24" t="str">
-        <x:v>Bend en vibrato word hoorbaar en diagnosties gemeet</x:v>
+        <x:v>Per-kanaal bend/CC1 diagnosties groen; hoorbare toets wag op US-016 en US-063</x:v>
       </x:c>
       <x:c r="L14" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-010</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-010 / v0.11.0</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="38" customHeight="1">
@@ -3607,13 +3607,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F66" s="83" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>Impediment</x:v>
       </x:c>
       <x:c r="G66" s="83" t="str">
         <x:v>Sprint 4</x:v>
       </x:c>
       <x:c r="H66" s="83" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Host ready / HIL blocked</x:v>
       </x:c>
       <x:c r="I66" s="83" t="n">
         <x:v>8</x:v>
@@ -3622,10 +3622,10 @@
         <x:v>US-006, US-007, US-052</x:v>
       </x:c>
       <x:c r="K66" s="83" t="str">
-        <x:v>BLE-bord ontvang Note/CC/bend via dieselfde eventmodel; S2 rapporteer unsupported sonder USB-regressie</x:v>
+        <x:v>S2 faal veilig sonder BLE; gedeelde transport groen; positiewe BLE-HIL wag op werklike BLE-bord</x:v>
       </x:c>
       <x:c r="L66" s="83" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / SCOPE-AMENDMENT-002 / MCP-US-062</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-062 / commit 535fde5</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
@@ -3704,7 +3704,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3e3d764672a4cc1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8600634f52144dea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3791,7 +3791,7 @@
       </x:c>
       <x:c r="E6" s="65" t="n">
         <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A6,'Backlog'!$F$5:$F$67,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F6" s="24" t="str">
         <x:v>USB, BLE en DIN/UART MIDI; guitar slides, kontroles en clock</x:v>
@@ -3942,7 +3942,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf5bb9abc139478f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02e63f5356c0443a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4687,7 +4687,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc717d7f66f84f60"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9957f557d1c418f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4861,7 +4861,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47293a240c0d4c6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28763a16aa174582"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5313,7 +5313,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b01c456ef54445b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fef0399e85f4b84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record MIDI batch host acceptance
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R015eca3c5ae74f88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R8289e600bf5b4c7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rce8f7e1e88894285"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rcbe5280a3ef84e7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Ra56ed1de19954598"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rb5c5ef7e31b64058"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Reaa43e3a31cb447c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R282f26b245f2460f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R4b0b20c314694bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Re5ecf69b40aa4aed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Rb61a977f68784ce0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R49aca2328e7a4b21"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -980,7 +980,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 2 | scope v0.13.0 | runtime v0.11.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 2 | scope v0.14.0 | runtime v0.11.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1039,7 +1039,7 @@
       </x:c>
       <x:c r="B6" s="114" t="n">
         <x:f>COUNTIF('Backlog'!$F$5:$F$67,"Done")</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
@@ -1138,7 +1138,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>Aktiewe hek: MCP-US-010 hoorbare bend/CC1 wag op I2S + D1 core | US-062 BLE HIL impediment | 68 hosttoetse groen</x:v>
+        <x:v>Host accepted: 68 passed + bend/CC1 + S2-negatiewe BLE | Device connection PASS | volume/deploy/klank/BLE-HIL bly oop</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1160,7 +1160,7 @@
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" s="123" t="str">
-        <x:v>Product Owner note: outonome hoststories is gepush. Fisiese USB/BLE/klank-aanvaarding bly menslike HIL en word nie uit hosttoetse afgelei nie.</x:v>
+        <x:v>Product Owner note 2026-07-15: hostbatch aanvaar. MCP-US-006 Done; fisiese USB, positiewe BLE en hoorbare klank bly aparte HIL-hekke.</x:v>
       </x:c>
       <x:c r="B15" s="124"/>
       <x:c r="C15" s="124"/>
@@ -1479,13 +1479,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F10" s="24" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G10" s="24" t="str">
         <x:v>Sprint 2</x:v>
       </x:c>
       <x:c r="H10" s="24" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I10" s="65" t="n">
         <x:v>5</x:v>
@@ -1494,10 +1494,10 @@
         <x:v>US-002</x:v>
       </x:c>
       <x:c r="K10" s="24" t="str">
-        <x:v>Note, CC, 14-bit bend en kanaallose clock gebruik backend-onafhanklike klasse; 49 hosttoetse en events-diagnose is groen</x:v>
+        <x:v>Product Owner het die draagbare eventmodel binne 68 groen hosttoetse aanvaar</x:v>
       </x:c>
       <x:c r="L10" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-006 / v0.6.0</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / HOST-ACCEPTED / v0.11.0</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="38" customHeight="1">
@@ -1523,7 +1523,7 @@
         <x:v>Sprint 2</x:v>
       </x:c>
       <x:c r="H11" s="24" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Host accepted / HIL pending</x:v>
       </x:c>
       <x:c r="I11" s="65" t="n">
         <x:v>5</x:v>
@@ -1532,10 +1532,10 @@
         <x:v>US-003, US-006</x:v>
       </x:c>
       <x:c r="K11" s="24" t="str">
-        <x:v>Host receive-loop groen; fisiese USB-MIDI Note On/Off wag op herstelbare toestel-deploy</x:v>
+        <x:v>Host receive-loop aanvaar; fisiese USB-MIDI Note On/Off wag op gemonteerde volume en deploy</x:v>
       </x:c>
       <x:c r="L11" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007 / commit 3ffc1bc</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007 / HOST-ACCEPTED</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
@@ -1637,7 +1637,7 @@
         <x:v>Sprint 2</x:v>
       </x:c>
       <x:c r="H14" s="24" t="str">
-        <x:v>Control ready / audible blocked</x:v>
+        <x:v>Host accepted / audible blocked</x:v>
       </x:c>
       <x:c r="I14" s="65" t="n">
         <x:v>5</x:v>
@@ -1646,10 +1646,10 @@
         <x:v>US-007</x:v>
       </x:c>
       <x:c r="K14" s="24" t="str">
-        <x:v>Per-kanaal bend/CC1 diagnosties groen; hoorbare toets wag op US-016 en US-063</x:v>
+        <x:v>Per-kanaal bend/CC1-berekening aanvaar; hoorbare toets wag op US-016 en US-063</x:v>
       </x:c>
       <x:c r="L14" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-010 / v0.11.0</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-010 / HOST-ACCEPTED</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="38" customHeight="1">
@@ -3613,7 +3613,7 @@
         <x:v>Sprint 4</x:v>
       </x:c>
       <x:c r="H66" s="83" t="str">
-        <x:v>Host ready / HIL blocked</x:v>
+        <x:v>S2 negative accepted / BLE HIL blocked</x:v>
       </x:c>
       <x:c r="I66" s="83" t="n">
         <x:v>8</x:v>
@@ -3622,10 +3622,10 @@
         <x:v>US-006, US-007, US-052</x:v>
       </x:c>
       <x:c r="K66" s="83" t="str">
-        <x:v>S2 faal veilig sonder BLE; gedeelde transport groen; positiewe BLE-HIL wag op werklike BLE-bord</x:v>
+        <x:v>S2-negatiewe gate aanvaar; positiewe BLE-HIL wag op 'n werklike BLE-bord</x:v>
       </x:c>
       <x:c r="L66" s="83" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-062 / commit 535fde5</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-062 / S2-NEGATIVE-ACCEPTED</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="48" customHeight="1">
@@ -3704,7 +3704,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8600634f52144dea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61db6e1c123a466f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3791,7 +3791,7 @@
       </x:c>
       <x:c r="E6" s="65" t="n">
         <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A6,'Backlog'!$F$5:$F$67,"Done")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F6" s="24" t="str">
         <x:v>USB, BLE en DIN/UART MIDI; guitar slides, kontroles en clock</x:v>
@@ -3942,7 +3942,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02e63f5356c0443a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84ee5940d15e4201"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4687,7 +4687,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9957f557d1c418f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R762296237c4c4067"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4861,7 +4861,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28763a16aa174582"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8828e674c1a54109"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5313,7 +5313,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fef0399e85f4b84"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92c12678cba8443a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(hil): close CircuitPython deployment dependencies
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Reaa43e3a31cb447c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R282f26b245f2460f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R4b0b20c314694bd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Re5ecf69b40aa4aed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Rb61a977f68784ce0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R49aca2328e7a4b21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcc9bd9a0a564457f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rb10292f5dbf047d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rd6d22c8563f146ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R21affbb057004ce8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R6880bb6d41534f4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rb401ff9078fa42d8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -750,7 +750,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Bron"/>
     <x:tableColumn id="2" name="Gebruik"/>
@@ -980,7 +980,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 2 | scope v0.14.0 | runtime v0.11.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 2 | scope v0.15.0 | runtime v0.11.1 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1138,7 +1138,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>Host accepted: 68 passed + bend/CC1 + S2-negatiewe BLE | Device connection PASS | volume/deploy/klank/BLE-HIL bly oop</x:v>
+        <x:v>82 tests GREEN | Wemos HIL: closure, 16 hashes, libraries, boot en imports PASS | USB-note/klank/BLE bly oop</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1160,7 +1160,7 @@
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" s="123" t="str">
-        <x:v>Product Owner note 2026-07-15: hostbatch aanvaar. MCP-US-006 Done; fisiese USB, positiewe BLE en hoorbare klank bly aparte HIL-hekke.</x:v>
+        <x:v>Product Owner note 2026-07-15: QA-herstel goedgekeur. Dependency-closed device proof PASS; US-007 Note On/Off bly oop.</x:v>
       </x:c>
       <x:c r="B15" s="124"/>
       <x:c r="C15" s="124"/>
@@ -1456,10 +1456,10 @@
         <x:v>US-003</x:v>
       </x:c>
       <x:c r="K9" s="24" t="str">
-        <x:v>Publieke verstekke, private settings en override-prioriteit is host-groen; toestel-deploy wag op leesalleen-volume herstel</x:v>
+        <x:v>Hostlektoetse is groen en die konfigurasielaag laai fisies; menslike private SET/UNSET-aanvaarding bly oop</x:v>
       </x:c>
       <x:c r="L9" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-005 / v0.5.0</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-051-IMP-001 / v0.11.1</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
@@ -1532,10 +1532,10 @@
         <x:v>US-003, US-006</x:v>
       </x:c>
       <x:c r="K11" s="24" t="str">
-        <x:v>Host receive-loop aanvaar; fisiese USB-MIDI Note On/Off wag op gemonteerde volume en deploy</x:v>
+        <x:v>Dependency-closed device deploy, harde boot en clean imports is fisies groen; werklike USB-MIDI Note On/Off bly oop</x:v>
       </x:c>
       <x:c r="L11" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007 / HOST-ACCEPTED</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-051-IMP-001 / v0.11.1</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
@@ -3204,10 +3204,10 @@
         <x:v>US-003, US-015</x:v>
       </x:c>
       <x:c r="K55" s="24" t="str">
-        <x:v>Connection/deploy/boot/execution-runner is groen; USB-MIDI bewys; klankmeting wag op US-015/016</x:v>
+        <x:v>Autoreload-safe deploy, closure, 16 hashes, libraries, boot en import/execution is fisies groen; klankadapter bly oop</x:v>
       </x:c>
       <x:c r="L55" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-051-IN-REVIEW</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-051-IMP-001 / v0.11.1</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="38" customHeight="1">
@@ -3704,7 +3704,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61db6e1c123a466f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd9907143572430e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3942,7 +3942,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84ee5940d15e4201"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf468f8966db645bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3967,7 +3967,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>29 geregistreerde risiko's; US-005 deploy is veilig gestop by 'n leesalleen CIRCUITPY-volume</x:v>
+        <x:v>29 geregistreerde risiko's; dependency-closed Wemos HIL slaag en R-029 is beheers</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -4332,7 +4332,7 @@
         <x:v>QA/Release</x:v>
       </x:c>
       <x:c r="F19" s="24" t="str">
-        <x:v>Backup, manifest en dry-run</x:v>
+        <x:v>Backup; dependency-closed 16-lêer manifest; nie-destruktiewe deploy; hash- en import-proof</x:v>
       </x:c>
       <x:c r="G19" s="24" t="str">
         <x:v>Controlled</x:v>
@@ -4657,7 +4657,7 @@
         <x:v>Stop deploy; FAT verify; fisiese power-cycle en skryfbaarheidstoets; geen erase/remount-omseiling</x:v>
       </x:c>
       <x:c r="G33" t="str">
-        <x:v>Open - US-005 HIL gate</x:v>
+        <x:v>Controlled - writable HIL 2026-07-15</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4687,7 +4687,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R762296237c4c4067"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd7cfb43d3d4433b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4861,7 +4861,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8828e674c1a54109"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7feade596b594f1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5087,7 +5087,7 @@
         <x:v>CircuitPython supervisor</x:v>
       </x:c>
       <x:c r="B18" t="str">
-        <x:v>USB-identiteit en runtime-inspeksie</x:v>
+        <x:v>USB ID, runtime, autoreload en hard reset</x:v>
       </x:c>
       <x:c r="C18" t="str">
         <x:v>Official API</x:v>
@@ -5304,6 +5304,20 @@
       </x:c>
       <x:c r="D33" t="str">
         <x:v>https://midi.org/summary-of-midi-1-0-messages</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" t="str">
+        <x:v>CircUp</x:v>
+      </x:c>
+      <x:c r="B34" t="str">
+        <x:v>Requirements-gebaseerde CircuitPython library-installering</x:v>
+      </x:c>
+      <x:c r="C34" t="str">
+        <x:v>Official tool</x:v>
+      </x:c>
+      <x:c r="D34" t="str">
+        <x:v>https://docs.circuitpython.org/projects/circup/en/latest/</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5313,7 +5327,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92c12678cba8443a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f8af9ccb27d458c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(config): normalize blank private settings
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb8e38f804be04039"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rcf916219bc8641a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rc7a906f9c37e435e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R1b532a9c79824ae0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R499be382f72846de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Re63355a4f39d49fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra7181de9364244f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R3055ec9c060242f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Re31549d4d9684c14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R6aa36888d4544ece"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Rb62c8d93eb664a26"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rfdeb6f5bbf9b4941"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -154,7 +154,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="22">
+  <x:fills count="25">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -261,6 +261,21 @@
         <x:fgColor rgb="FF80C6E3"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFBFE5F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE0D1"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="8">
     <x:border/>
@@ -333,7 +348,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="137">
+  <x:cellXfs count="140">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -667,6 +682,15 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1036,7 +1060,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 2 | scope v0.16.0 | runtime v0.12.2 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 2 | scope v0.17.0 | runtime v0.12.3 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1078,7 +1102,7 @@
       </x:c>
       <x:c r="B5" s="113" t="n">
         <x:f>COUNTA('Backlog'!$A$5:$A$200)</x:f>
-        <x:v>68</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="C5" s="85"/>
       <x:c r="D5" s="110" t="str">
@@ -1146,7 +1170,7 @@
       </x:c>
       <x:c r="B9" s="114" t="n">
         <x:f>COUNTA('Risks'!$A$5:$A$200)</x:f>
-        <x:v>30</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C9" s="85"/>
       <x:c r="D9" s="116" t="str">
@@ -1194,7 +1218,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>89 tests GREEN | Wemos HIL: closure, libraries, boot, imports en USB Note On/Off PASS | audio/BLE bly oop</x:v>
+        <x:v>91 tests GREEN | USB-MIDI HIL PASS | US-005 leewaarde-herstel wag op finale Wemos-herbewys | audio/BLE bly oop</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1216,7 +1240,7 @@
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" s="123" t="str">
-        <x:v>Product Owner note 2026-07-15: MCP-US-007 aanvaar; matched USB-MIDI Note On/Off op S2 Mini. Framework Engineering baseline bygevoeg.</x:v>
+        <x:v>Product Owner note 2026-07-16: fisiese chip/display uitbreiding is post-MVP; US-023 besit hostname/IP startupstatus.</x:v>
       </x:c>
       <x:c r="B15" s="124"/>
       <x:c r="C15" s="124"/>
@@ -1288,7 +1312,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md | 68 stories | Redigeer Status en Priority via keuselyste</x:v>
+        <x:v>Bron: docs/user_stories_v0.1.0.md | 74 stories | Redigeer Status en Priority via keuselyste</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -1513,10 +1537,10 @@
         <x:v>US-003</x:v>
       </x:c>
       <x:c r="K9" s="24" t="str">
-        <x:v>Hostlektoetse is groen en die konfigurasielaag laai fisies; menslike private SET/UNSET-aanvaarding bly oop</x:v>
+        <x:v>Hostlek- en leewaarde-toetse is groen; Wemos moet leë/whitespace private settings as UNSET en ingevulde waardes slegs as SET rapporteer</x:v>
       </x:c>
       <x:c r="L9" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-051-IMP-001 / v0.11.1</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-005-RETEST / v0.12.3</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
@@ -2197,10 +2221,10 @@
         <x:v>US-005, US-022</x:v>
       </x:c>
       <x:c r="K27" s="24" t="str">
-        <x:v>Runtime join 'n gekonfigureerde netwerk binne timeout en rapporteer station-IP; by mislukking begin 'n beveiligde AP en rapporteer AP-IP sonder MIDI-/klankblokkasie</x:v>
+        <x:v>Startup rapporteer hostname plus station/IP of veilige AP-fallback/IP; join is begrens, geredigeer en blokkeer nie MIDI/klank nie</x:v>
       </x:c>
       <x:c r="L27" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / WIFI-RUNTIME-AMENDMENT-001 / MCP-US-023</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE-START / MCP-US-023</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="38" customHeight="1">
@@ -3911,6 +3935,234 @@
       </x:c>
       <x:c r="L72" s="126" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE / MCP-US-068</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="52" customHeight="1">
+      <x:c r="A73" s="137" t="str">
+        <x:v>MCP-US-069</x:v>
+      </x:c>
+      <x:c r="B73" s="137" t="str">
+        <x:v>MCP-EPIC-010</x:v>
+      </x:c>
+      <x:c r="C73" s="137" t="str">
+        <x:v>External I2C Status Display Adapter</x:v>
+      </x:c>
+      <x:c r="D73" s="137" t="str">
+        <x:v>Embedded/Web</x:v>
+      </x:c>
+      <x:c r="E73" s="137" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="F73" s="137" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G73" s="137" t="str">
+        <x:v>Post-MVP</x:v>
+      </x:c>
+      <x:c r="H73" s="137" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+      <x:c r="I73" s="137" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J73" s="137" t="str">
+        <x:v>US-004, US-022</x:v>
+      </x:c>
+      <x:c r="K73" s="137" t="str">
+        <x:v>Capability-gated SSD1306/similar display shows rate-limited status; absence never changes synth behavior</x:v>
+      </x:c>
+      <x:c r="L73" s="137" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE-START / MCP-US-069</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="52" customHeight="1">
+      <x:c r="A74" s="138" t="str">
+        <x:v>MCP-US-070</x:v>
+      </x:c>
+      <x:c r="B74" s="138" t="str">
+        <x:v>MCP-EPIC-010</x:v>
+      </x:c>
+      <x:c r="C74" s="138" t="str">
+        <x:v>Physical Chip Transport And Capability Abstraction</x:v>
+      </x:c>
+      <x:c r="D74" s="138" t="str">
+        <x:v>Solution Architect</x:v>
+      </x:c>
+      <x:c r="E74" s="138" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="F74" s="138" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G74" s="138" t="str">
+        <x:v>Post-MVP</x:v>
+      </x:c>
+      <x:c r="H74" s="138" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+      <x:c r="I74" s="138" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J74" s="138" t="str">
+        <x:v>US-004, US-034</x:v>
+      </x:c>
+      <x:c r="K74" s="138" t="str">
+        <x:v>Class-based GPIO, I2C-expander and SPI transport ports are capability-gated without chip or pin constants</x:v>
+      </x:c>
+      <x:c r="L74" s="138" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE-START / MCP-US-070</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="52" customHeight="1">
+      <x:c r="A75" s="137" t="str">
+        <x:v>MCP-US-071</x:v>
+      </x:c>
+      <x:c r="B75" s="137" t="str">
+        <x:v>MCP-EPIC-010</x:v>
+      </x:c>
+      <x:c r="C75" s="137" t="str">
+        <x:v>Physical SN76489 Hardware Adapter</x:v>
+      </x:c>
+      <x:c r="D75" s="137" t="str">
+        <x:v>DSP/Chip Engineer</x:v>
+      </x:c>
+      <x:c r="E75" s="137" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="F75" s="137" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G75" s="137" t="str">
+        <x:v>Post-MVP</x:v>
+      </x:c>
+      <x:c r="H75" s="137" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+      <x:c r="I75" s="137" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J75" s="137" t="str">
+        <x:v>US-017, US-070</x:v>
+      </x:c>
+      <x:c r="K75" s="137" t="str">
+        <x:v>Verified chip identity, levels, clock and bus sequences drive hardware; failures fall back to emulation</x:v>
+      </x:c>
+      <x:c r="L75" s="137" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE-START / MCP-US-071</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="52" customHeight="1">
+      <x:c r="A76" s="138" t="str">
+        <x:v>MCP-US-072</x:v>
+      </x:c>
+      <x:c r="B76" s="138" t="str">
+        <x:v>MCP-EPIC-010</x:v>
+      </x:c>
+      <x:c r="C76" s="138" t="str">
+        <x:v>Physical SID6581 Feasibility And Adapter</x:v>
+      </x:c>
+      <x:c r="D76" s="138" t="str">
+        <x:v>DSP/Chip Engineer</x:v>
+      </x:c>
+      <x:c r="E76" s="138" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="F76" s="138" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G76" s="138" t="str">
+        <x:v>Post-MVP</x:v>
+      </x:c>
+      <x:c r="H76" s="138" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+      <x:c r="I76" s="138" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="J76" s="138" t="str">
+        <x:v>US-038, US-070</x:v>
+      </x:c>
+      <x:c r="K76" s="138" t="str">
+        <x:v>Power, levels, clock, register bus and analog output receive a measured go/no-go before implementation</x:v>
+      </x:c>
+      <x:c r="L76" s="138" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE-START / MCP-US-072</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="52" customHeight="1">
+      <x:c r="A77" s="137" t="str">
+        <x:v>MCP-US-073</x:v>
+      </x:c>
+      <x:c r="B77" s="137" t="str">
+        <x:v>MCP-EPIC-010</x:v>
+      </x:c>
+      <x:c r="C77" s="137" t="str">
+        <x:v>ArduinoOPL2 SPI Hardware Adapter</x:v>
+      </x:c>
+      <x:c r="D77" s="137" t="str">
+        <x:v>DSP/Chip Engineer</x:v>
+      </x:c>
+      <x:c r="E77" s="137" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="F77" s="137" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G77" s="137" t="str">
+        <x:v>Post-MVP</x:v>
+      </x:c>
+      <x:c r="H77" s="137" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+      <x:c r="I77" s="137" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J77" s="137" t="str">
+        <x:v>US-041, US-070</x:v>
+      </x:c>
+      <x:c r="K77" s="137" t="str">
+        <x:v>DhrBaksteen SPI contract and license are reviewed and verified by real HIL without coupling bus and emulator logic</x:v>
+      </x:c>
+      <x:c r="L77" s="137" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE-START / MCP-US-073</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="52" customHeight="1">
+      <x:c r="A78" s="138" t="str">
+        <x:v>MCP-US-074</x:v>
+      </x:c>
+      <x:c r="B78" s="138" t="str">
+        <x:v>MCP-EPIC-010</x:v>
+      </x:c>
+      <x:c r="C78" s="138" t="str">
+        <x:v>Emulated Or Physical Core Backend Selection And Fallback</x:v>
+      </x:c>
+      <x:c r="D78" s="138" t="str">
+        <x:v>Solution Architect/DSP</x:v>
+      </x:c>
+      <x:c r="E78" s="138" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="F78" s="138" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G78" s="138" t="str">
+        <x:v>Post-MVP</x:v>
+      </x:c>
+      <x:c r="H78" s="138" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+      <x:c r="I78" s="138" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J78" s="138" t="str">
+        <x:v>US-034, US-070, one physical adapter</x:v>
+      </x:c>
+      <x:c r="K78" s="138" t="str">
+        <x:v>Config/web selects emulated or physical per core; emulation is default/fallback and physical mode avoids duplicate rendering</x:v>
+      </x:c>
+      <x:c r="L78" s="138" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE-START / MCP-US-074</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3951,7 +4203,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Read74dcd298d427b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ea335e9402f4f6c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4205,6 +4457,29 @@
         <x:v>Vision, architecture, meta model, quality and controlled agent context</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="48" customHeight="1">
+      <x:c r="A14" s="138" t="str">
+        <x:v>MCP-EPIC-010</x:v>
+      </x:c>
+      <x:c r="B14" s="138" t="str">
+        <x:v>Physical Chip And Display Expansion</x:v>
+      </x:c>
+      <x:c r="C14" s="138" t="n">
+        <x:f>COUNTIF('Backlog'!$B$5:$B$200,A14)</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D14" s="138" t="n">
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A14,'Backlog'!$E$5:$E$200,"Must")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E14" s="138" t="n">
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A14,'Backlog'!$F$5:$F$200,"Done")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F14" s="138" t="str">
+        <x:v>Post-MVP displays and physical SN76489/SID/OPL2 backends with emulation fallback</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
@@ -4212,7 +4487,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb2a5f040ee842a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd85fc2c2154d4954"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4237,7 +4512,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>30 geregistreerde risiko's; USB-MIDI HIL slaag en unieke instance-identiteit is as R-030 / US-068 georden</x:v>
+        <x:v>32 geregistreerde risiko's; fisiese-chip skade en backend-fallback is eksplisiet post-MVP beheer</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -4951,6 +5226,52 @@
       </x:c>
       <x:c r="G34" s="126" t="str">
         <x:v>Backlog - US-068</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="48" customHeight="1">
+      <x:c r="A35" s="139" t="str">
+        <x:v>R-031</x:v>
+      </x:c>
+      <x:c r="B35" s="139" t="str">
+        <x:v>Wrong power, levels, clock or bus sequence damages a rare physical retro chip</x:v>
+      </x:c>
+      <x:c r="C35" s="139" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="D35" s="139" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="E35" s="139" t="str">
+        <x:v>DSP/Chip/Hardware</x:v>
+      </x:c>
+      <x:c r="F35" s="139" t="str">
+        <x:v>Datasheet and measurement gate, current-limited supply, level shifting and no universal expander assumption</x:v>
+      </x:c>
+      <x:c r="G35" s="139" t="str">
+        <x:v>Later - US-070 to US-073</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="48" customHeight="1">
+      <x:c r="A36" s="138" t="str">
+        <x:v>R-032</x:v>
+      </x:c>
+      <x:c r="B36" s="138" t="str">
+        <x:v>Physical backend is falsely detected, hangs runtime or plays alongside emulation</x:v>
+      </x:c>
+      <x:c r="C36" s="138" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="D36" s="138" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E36" s="138" t="str">
+        <x:v>Architect/Embedded/QA</x:v>
+      </x:c>
+      <x:c r="F36" s="138" t="str">
+        <x:v>Capability probe, timeout, fault injection, safe switch boundary and emulation default/fallback</x:v>
+      </x:c>
+      <x:c r="G36" s="138" t="str">
+        <x:v>Later - US-074</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4980,7 +5301,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d478ddd7fdf482c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e19665bb2134742"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5176,7 +5497,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21e91df7a89d4cc0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb18fc9a79c14d0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5635,6 +5956,34 @@
         <x:v>https://docs.circuitpython.org/projects/circup/en/latest/</x:v>
       </x:c>
     </x:row>
+    <x:row r="35" ht="44" customHeight="1">
+      <x:c r="A35" s="137" t="str">
+        <x:v>DhrBaksteen ArduinoOPL2</x:v>
+      </x:c>
+      <x:c r="B35" s="137" t="str">
+        <x:v>Later OPL2 SPI contract, license and HIL</x:v>
+      </x:c>
+      <x:c r="C35" s="137" t="str">
+        <x:v>User-provided source</x:v>
+      </x:c>
+      <x:c r="D35" s="137" t="str">
+        <x:v>https://github.com/DhrBaksteen/ArduinoOPL2/tree/master/src</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="44" customHeight="1">
+      <x:c r="A36" s="138" t="str">
+        <x:v>Malvineous pyopl</x:v>
+      </x:c>
+      <x:c r="B36" s="138" t="str">
+        <x:v>Later OPL2 behavior and test reference</x:v>
+      </x:c>
+      <x:c r="C36" s="138" t="str">
+        <x:v>User-provided source</x:v>
+      </x:c>
+      <x:c r="D36" s="138" t="str">
+        <x:v>https://github.com/Malvineous/pyopl</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -5642,7 +5991,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ad94215b7fc4528"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5a4edd19c644ba6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(qa): add burn-in and heap leak gates
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R35f4bc40367241cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Ra81e651c4a134d3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R390e254c652b43c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Re1ab7c876df64e1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R5ee93503758a4f2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R7ca07df745f14431"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R56b233f66fba4e1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Ra1d0771eb73a43dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R445bdf1523bb49e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rb56cdf5a2d7a4a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R90850cbbf8164d8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R73876813407642e1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -154,7 +154,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="27">
+  <x:fills count="29">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -286,6 +286,16 @@
         <x:fgColor rgb="FFFCE0D1"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE0D1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="8">
     <x:border/>
@@ -358,7 +368,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="143">
+  <x:cellXfs count="145">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -710,6 +720,12 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1079,7 +1095,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 2 | scope v0.18.0 | runtime v0.12.3 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 2 | scope v0.19.0 | runtime v0.12.3 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1189,7 +1205,7 @@
       </x:c>
       <x:c r="B9" s="114" t="n">
         <x:f>COUNTA('Risks'!$A$5:$A$200)</x:f>
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C9" s="85"/>
       <x:c r="D9" s="116" t="str">
@@ -1237,7 +1253,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>91 tests GREEN | USB-MIDI HIL PASS | US-005 UNSET-HIL wag | volgende: AudioOutput -&gt; standalone I2S -&gt; D1 -&gt; Logic</x:v>
+        <x:v>91 tests GREEN | USB-MIDI HIL PASS | US-005 UNSET-HIL wag | D1 MVP vereis 8h audio/heap burn-in</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1332,7 +1348,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md v0.18.0 | 74 stories | 16-story bevrore MVP Acceptance Set</x:v>
+        <x:v>Bron: docs/user_stories_v0.1.0.md v0.19.0 | 74 stories | 16-story bevrore MVP Acceptance Set</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -1975,7 +1991,7 @@
         <x:v>US-004, US-014</x:v>
       </x:c>
       <x:c r="K20" s="24" t="str">
-        <x:v>Class-based device/i2s_test.py imports no synth package or global state; injected PCM-I2S profile plays G3-C4-D4 square waves; MAX98357 IO5/IO3/IO7 passes audible HIL and releases I2S</x:v>
+        <x:v>Class-based device/i2s_test.py imports no synth package/global state; G3-C4-D4 square waves pass MAX98357 HIL, release I2S and complete a 30-minute smoke</x:v>
       </x:c>
       <x:c r="L20" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MVP-SCOPE-REDUCTION-001 / MCP-US-016</x:v>
@@ -3305,7 +3321,7 @@
         <x:v>US-003, US-016</x:v>
       </x:c>
       <x:c r="K55" s="24" t="str">
-        <x:v>Deploy/closure/boot/import execution remains green; MAX98357 audio adapter closes with US-016 audible proof</x:v>
+        <x:v>Deploy/closure/boot/import execution remains green; audio adapter adds rate-limited heap, reset and dropout burn-in telemetry</x:v>
       </x:c>
       <x:c r="L55" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-051-IMP-001 / v0.11.1</x:v>
@@ -3457,7 +3473,7 @@
         <x:v>US-003, US-007, US-009, US-014, US-016, US-063</x:v>
       </x:c>
       <x:c r="K59" s="24" t="str">
-        <x:v>Logic selects the board as External MIDI, sends Note On/Off and the user hears D1 through the reference I2S path</x:v>
+        <x:v>Logic selects the board and the user hears D1; the reference board then passes an 8-hour USB-MIDI/audio/heap burn-in</x:v>
       </x:c>
       <x:c r="L59" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-055</x:v>
@@ -3533,7 +3549,7 @@
         <x:v>US-001 to US-009, US-014, US-016, US-050, US-051, US-055, US-063</x:v>
       </x:c>
       <x:c r="K61" s="25" t="str">
-        <x:v>Tag, release notes and known limitations accompany a repeatable Logic USB-MIDI to audible D1 demo</x:v>
+        <x:v>Tag, release notes, known limitations and a passing 8-hour burn-in report accompany the Logic-to-audible-D1 demo</x:v>
       </x:c>
       <x:c r="L61" s="25" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-057</x:v>
@@ -3761,7 +3777,7 @@
         <x:v>US-006, US-008, US-009, US-014, US-016</x:v>
       </x:c>
       <x:c r="K67" s="83" t="str">
-        <x:v>Portable sine/saw/square D1 handles Note On/Off through AudioOutput; no desktop backend or production-repo modification</x:v>
+        <x:v>Portable sine/saw/square D1 handles Note On/Off, cleans up and passes a 30-minute smoke; no production-repo modification</x:v>
       </x:c>
       <x:c r="L67" s="83" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / SCOPE-AMENDMENT-002 / MCP-US-063</x:v>
@@ -4223,7 +4239,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82a0242ac61e4764"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29b4a5407aa04305"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4507,7 +4523,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f8ff8dc40e04d41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fae457530fd4d62"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4532,7 +4548,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>33 geregistreerde risiko's; onafhanklike I2S-diagnose se profiel-drift word eksplisiet beheer</x:v>
+        <x:v>34 geregistreerde risiko's; I2S-profieldrift en langdurige heap/resource-lekke word eksplisiet beheer</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -5295,26 +5311,49 @@
       </x:c>
     </x:row>
     <x:row r="37" ht="48" customHeight="1">
-      <x:c r="A37" s="142" t="str">
+      <x:c r="A37" s="143" t="str">
         <x:v>R-033</x:v>
       </x:c>
-      <x:c r="B37" s="142" t="str">
+      <x:c r="B37" s="143" t="str">
         <x:v>Standalone I2S diagnostic drifts from the production AudioOutput profile</x:v>
       </x:c>
-      <x:c r="C37" s="142" t="str">
+      <x:c r="C37" s="143" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="D37" s="142" t="str">
+      <x:c r="D37" s="143" t="str">
         <x:v>High</x:v>
       </x:c>
-      <x:c r="E37" s="142" t="str">
+      <x:c r="E37" s="143" t="str">
         <x:v>Architect/QA/HIL</x:v>
       </x:c>
-      <x:c r="F37" s="142" t="str">
+      <x:c r="F37" s="143" t="str">
         <x:v>Same profile field names, AST/import and frequency tests, paired MAX98357 HIL, no shared synth-runtime import</x:v>
       </x:c>
-      <x:c r="G37" s="142" t="str">
+      <x:c r="G37" s="143" t="str">
         <x:v>Controlled in US-016</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="48" customHeight="1">
+      <x:c r="A38" s="144" t="str">
+        <x:v>R-034</x:v>
+      </x:c>
+      <x:c r="B38" s="144" t="str">
+        <x:v>Long-running heap/resource leak or rare reset is missed by short HIL</x:v>
+      </x:c>
+      <x:c r="C38" s="144" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="D38" s="144" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E38" s="144" t="str">
+        <x:v>QA/HIL/Embedded</x:v>
+      </x:c>
+      <x:c r="F38" s="144" t="str">
+        <x:v>30m/8h/12h/24h burn-in profiles, 4096-byte/5% heap boundary, cleanup/reset/dropout telemetry</x:v>
+      </x:c>
+      <x:c r="G38" s="144" t="str">
+        <x:v>Controlled in US-016/051/055/057</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5344,7 +5383,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45f9eabe879e4fa5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9110a836be354f5a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5540,7 +5579,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb203d2a4fb04fdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b713b665a2c4402"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6034,7 +6073,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R175a54341c2e4e9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R418affa2b07b4c66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(us005): record configuration HIL acceptance
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R56b233f66fba4e1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Ra1d0771eb73a43dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R445bdf1523bb49e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rb56cdf5a2d7a4a05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R90850cbbf8164d8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R73876813407642e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf6f88ae00d934a50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R1b3f7cd50645453a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R400cdd6a1f3e4cdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R135db6911b98465d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R1089bb58a2874c1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R36160fdbbe1045f7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1095,7 +1095,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 2 | scope v0.19.0 | runtime v0.12.3 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 2 | scope v0.20.0 | runtime v0.12.3 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1141,7 +1141,7 @@
       </x:c>
       <x:c r="C5" s="85"/>
       <x:c r="D5" s="110" t="str">
-        <x:v>1. Sluit US-005 SET/UNSET-konfigurasiegrens</x:v>
+        <x:v>1. US-005 config/geheimegrens fisies aanvaar</x:v>
       </x:c>
       <x:c r="E5" s="110"/>
       <x:c r="F5" s="110"/>
@@ -1154,11 +1154,11 @@
       </x:c>
       <x:c r="B6" s="114" t="n">
         <x:f>COUNTIF('Backlog'!$F$5:$F$200,"Done")</x:f>
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
-        <x:v>2. Bou AudioOutput en onafhanklike G-C-D I2S-preflight</x:v>
+        <x:v>2. Bou US-014 AudioOutput; daarna US-016 G-C-D I2S-preflight</x:v>
       </x:c>
       <x:c r="E6" s="111"/>
       <x:c r="F6" s="111"/>
@@ -1253,7 +1253,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>91 tests GREEN | USB-MIDI HIL PASS | US-005 UNSET-HIL wag | D1 MVP vereis 8h audio/heap burn-in</x:v>
+        <x:v>91 tests GREEN | USB-MIDI HIL PASS | US-005 UNSET-HIL PASS | aktief: US-014 AudioOutput</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1348,7 +1348,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md v0.19.0 | 74 stories | 16-story bevrore MVP Acceptance Set</x:v>
+        <x:v>Bron: docs/user_stories_v0.1.0.md v0.20.0 | 74 stories | 16-story bevrore MVP Acceptance Set</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -1558,13 +1558,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F9" s="24" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G9" s="24" t="str">
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H9" s="24" t="str">
-        <x:v>MVP-Enabler (In Review)</x:v>
+        <x:v>MVP-Enabler (Done)</x:v>
       </x:c>
       <x:c r="I9" s="65" t="n">
         <x:v>5</x:v>
@@ -1573,10 +1573,10 @@
         <x:v>US-003</x:v>
       </x:c>
       <x:c r="K9" s="24" t="str">
-        <x:v>Hostlek- en leewaarde-toetse is groen; Wemos moet leë/whitespace private settings as UNSET en ingevulde waardes slegs as SET rapporteer</x:v>
+        <x:v>Host secret-leak tests and Wemos v0.12.3 prove PASS, three empty private settings as UNSET and device execution READY without exposing values</x:v>
       </x:c>
       <x:c r="L9" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-005-RETEST / v0.12.3</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-005-HIL-ACCEPTED</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
@@ -4239,7 +4239,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29b4a5407aa04305"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76654acddac14138"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4303,7 +4303,7 @@
       </x:c>
       <x:c r="E5" s="64" t="n">
         <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A5,'Backlog'!$F$5:$F$200,"Done")</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F5" s="23" t="str">
         <x:v>MVP enablers: safe boot, board profile and configuration boundary</x:v>
@@ -4523,7 +4523,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fae457530fd4d62"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c3d1fa5b71d4541"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5383,7 +5383,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9110a836be354f5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67be7e6abe204775"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5579,7 +5579,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b713b665a2c4402"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re29fbd01fe714688"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6073,7 +6073,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R418affa2b07b4c66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree582e3e91704933"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>